<commit_message>
Metals: gold ETFs and central-bank purchases (World Gold Council)
New sub-tab with ETF holdings, demand and flows by region since 2003 against
the price, the largest funds, net central-bank buying by month, top buyers and
sellers, and one country's history. The metals desk read now gets these too.
The owner can upload the monthly Goldhub files from the tab; uploads live
next to the database and survive deploys. Holdings file updated to Oct 2026.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/refdata/wgc_official_gold_holdings.xlsx
+++ b/refdata/wgc_official_gold_holdings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://worldgoldcouncil.sharepoint.com/sites/ResearchStrategy/Shared Documents/Central bank stats/2026/Aug/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://worldgoldcouncil.sharepoint.com/sites/ResearchStrategy/Shared Documents/Central bank stats/2026/Oct/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="8_{5692D4FD-4F4C-480F-8444-CBBDF161C826}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{05C6A9F2-F019-499C-A7F1-61F1428E6A7C}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="8_{1F691327-9DAE-46DA-BFB9-E30DD01EE949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE882F2E-9B5C-4C5D-87FF-B2733520375F}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" xr2:uid="{3523EF29-3059-43FF-81DC-EB23E42866DD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="17520" xr2:uid="{4F59338A-933D-4B54-A59B-7F9911D93ED4}"/>
   </bookViews>
   <sheets>
     <sheet name="PDF" sheetId="1" r:id="rId1"/>
@@ -76,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="118">
   <si>
     <t>WORLD OFFICIAL GOLD HOLDINGS</t>
   </si>
@@ -99,6 +99,9 @@
     <t>Euro Area (incl. ECB)</t>
   </si>
   <si>
+    <t>International Financial Statistics, October 2026*</t>
+  </si>
+  <si>
     <t>United States</t>
   </si>
   <si>
@@ -138,15 +141,15 @@
     <t>Russian Federation</t>
   </si>
   <si>
+    <t>Malaysia</t>
+  </si>
+  <si>
+    <t>Switzerland</t>
+  </si>
+  <si>
     <t>Finland</t>
   </si>
   <si>
-    <t>Switzerland</t>
-  </si>
-  <si>
-    <t>Malaysia</t>
-  </si>
-  <si>
     <t>India</t>
   </si>
   <si>
@@ -195,7 +198,7 @@
     <t>Ghana</t>
   </si>
   <si>
-    <t>Jun 2026</t>
+    <t>Aug 2026</t>
   </si>
   <si>
     <t>Portugal</t>
@@ -204,6 +207,9 @@
     <t>Bolivia</t>
   </si>
   <si>
+    <t>Jul 2026</t>
+  </si>
+  <si>
     <t>Kazakhstan, Rep. of</t>
   </si>
   <si>
@@ -270,15 +276,15 @@
     <t>Iraq</t>
   </si>
   <si>
+    <t>Chile</t>
+  </si>
+  <si>
+    <t>Algeria</t>
+  </si>
+  <si>
     <t>Curaçao and Sint Maarten</t>
   </si>
   <si>
-    <t>Algeria</t>
-  </si>
-  <si>
-    <t>Chile</t>
-  </si>
-  <si>
     <t>Brazil</t>
   </si>
   <si>
@@ -360,15 +366,15 @@
     <t>Bahrain, Kingdom of</t>
   </si>
   <si>
+    <t>Zimbabwe</t>
+  </si>
+  <si>
+    <t>Indonesia</t>
+  </si>
+  <si>
     <t>Brunei Darussalam</t>
   </si>
   <si>
-    <t>Indonesia</t>
-  </si>
-  <si>
-    <t>Zimbabwe</t>
-  </si>
-  <si>
     <t>Czech Rep.</t>
   </si>
   <si>
@@ -378,34 +384,31 @@
     <t>Australia</t>
   </si>
   <si>
-    <t>Mozambique, Rep. of</t>
+    <t>Albania</t>
   </si>
   <si>
     <t>Kuwait</t>
   </si>
   <si>
-    <t>Albania</t>
+    <t>Bosnia and Herzegovina</t>
+  </si>
+  <si>
+    <t>United Arab Emirates</t>
+  </si>
+  <si>
+    <t>Aruba, Kingdom of the Netherlands</t>
   </si>
   <si>
     <t>Jordan</t>
   </si>
   <si>
-    <t>Bosnia and Herzegovina</t>
-  </si>
-  <si>
-    <t>United Arab Emirates</t>
-  </si>
-  <si>
-    <t>Aruba, Kingdom of the Netherlands</t>
+    <t>Luxembourg</t>
   </si>
   <si>
     <t>Denmark</t>
   </si>
   <si>
-    <t>Luxembourg</t>
-  </si>
-  <si>
-    <t>International Financial Statistics, August 2026*</t>
+    <t>El Salvador</t>
   </si>
   <si>
     <r>
@@ -454,7 +457,7 @@
   </si>
   <si>
     <r>
-      <t>Belarus, Rep. of</t>
+      <t>Belarus, Rep. o</t>
     </r>
     <r>
       <rPr>
@@ -464,7 +467,7 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t>4)</t>
+      <t>f4)</t>
     </r>
   </si>
   <si>
@@ -683,10 +686,10 @@
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{99AEFD7F-039D-4153-8082-67E70274AFFD}"/>
-    <cellStyle name="Normal 3" xfId="2" xr:uid="{BA18A9DE-A546-4F06-AA41-C509579CCA8E}"/>
-    <cellStyle name="Percent 2 2" xfId="4" xr:uid="{7D4FE88A-0650-4150-9621-D2DA9BCE6243}"/>
-    <cellStyle name="Percent 3" xfId="3" xr:uid="{3FB98E87-7F85-4F2C-A504-62061D1887DC}"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{7465BB16-A4E3-449D-BC78-268B1E02BD82}"/>
+    <cellStyle name="Normal 3" xfId="2" xr:uid="{E411E35E-6D7D-4FD6-B1C3-36DD044E889D}"/>
+    <cellStyle name="Percent 2 2" xfId="4" xr:uid="{CCEF6B80-052A-4360-97C9-E4434DDC96CB}"/>
+    <cellStyle name="Percent 3" xfId="3" xr:uid="{E3DE2B33-5066-47AB-9C8B-0DC849136578}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -721,7 +724,7 @@
         <xdr:cNvPr id="2" name="Text Box 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{59BCFD74-8EE5-4E2C-8392-E2C69319EBBA}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{69B6DA8B-875C-4A76-AE2C-F3EC0415988D}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -731,8 +734,8 @@
       </xdr:nvSpPr>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="603250" y="11753849"/>
-          <a:ext cx="6508750" cy="7429500"/>
+          <a:off x="600075" y="11563349"/>
+          <a:ext cx="6496050" cy="7286625"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -783,7 +786,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>August</a:t>
+            <a:t>October</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="en-GB" sz="1000" b="1" i="0" baseline="0">
@@ -818,7 +821,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>August 2026 </a:t>
+            <a:t>October 2026 </a:t>
           </a:r>
           <a:r>
             <a:rPr lang="en-GB" sz="1000" b="0" i="0" baseline="0">
@@ -834,7 +837,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>June 2026 </a:t>
+            <a:t>August 2026 </a:t>
           </a:r>
           <a:r>
             <a:rPr lang="en-GB" sz="1000" b="0" i="0" baseline="0">
@@ -850,7 +853,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>May 2026 </a:t>
+            <a:t>July 2026 </a:t>
           </a:r>
           <a:r>
             <a:rPr lang="en-GB" sz="1000" b="0" i="0" baseline="0">
@@ -885,7 +888,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>June 2026 </a:t>
+            <a:t>August 2026 </a:t>
           </a:r>
           <a:r>
             <a:rPr lang="en-GB" sz="1000" b="0" i="0" baseline="0">
@@ -901,7 +904,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>US$4026.05/oz</a:t>
+            <a:t>US$4562.75/oz</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="en-GB" sz="1000" b="0" i="0" baseline="0">
@@ -1284,7 +1287,7 @@
         <xdr:cNvPr id="3" name="Text Box 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A1A6D604-36B2-4245-9676-27A8502A1BBA}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B005B68D-2CA8-4F87-B617-2603065A3270}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1294,8 +1297,8 @@
       </xdr:nvSpPr>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="260350" y="20516850"/>
-          <a:ext cx="7340600" cy="6908800"/>
+          <a:off x="257175" y="20154900"/>
+          <a:ext cx="7324725" cy="6781800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1839,7 +1842,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B0DD703-EC2F-4317-AC11-9D185CAADF7E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB3C0268-7D72-42CB-AADA-4412A794437C}">
   <sheetPr codeName="Sheet6"/>
   <dimension ref="A3:O146"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
@@ -1875,7 +1878,7 @@
     </row>
     <row r="4" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="34" t="s">
-        <v>109</v>
+        <v>7</v>
       </c>
       <c r="B4" s="34"/>
       <c r="C4" s="34"/>
@@ -1929,31 +1932,31 @@
         <v>1</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C7" s="7">
         <v>8133.4616727317971</v>
       </c>
       <c r="D7" s="8">
-        <v>0.81421861947241103</v>
+        <v>0.83033510459195603</v>
       </c>
       <c r="E7" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="F7" s="1">
         <v>51</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H7" s="7">
         <v>64.823231227644555</v>
       </c>
       <c r="I7" s="8">
-        <v>0.2988200079124011</v>
+        <v>0.3396949332509645</v>
       </c>
       <c r="J7" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="K7" s="7"/>
     </row>
@@ -1962,31 +1965,31 @@
         <v>2</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C8" s="7">
-        <v>3349.4759105471057</v>
+        <v>3349.2892911573517</v>
       </c>
       <c r="D8" s="8">
-        <v>0.80993141992293249</v>
+        <v>0.82687917456518312</v>
       </c>
       <c r="E8" s="9">
-        <v>46142</v>
+        <v>46234</v>
       </c>
       <c r="F8" s="1">
         <v>52</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H8" s="7">
         <v>61.73873938602221</v>
       </c>
       <c r="I8" s="8">
-        <v>0.1789029731247137</v>
+        <v>0.18688392886663324</v>
       </c>
       <c r="J8" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="K8" s="7"/>
     </row>
@@ -1995,31 +1998,31 @@
         <v>3</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C9" s="7">
         <v>2814.0420826723898</v>
       </c>
       <c r="D9" s="35" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E9" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="F9" s="1">
         <v>53</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H9" s="7">
-        <v>57.300927302587795</v>
+        <v>57.30106680058163</v>
       </c>
       <c r="I9" s="8">
-        <v>0.29410055941702046</v>
+        <v>0.33049699119354015</v>
       </c>
       <c r="J9" s="9">
-        <v>46203</v>
+        <v>46234</v>
       </c>
       <c r="K9" s="7"/>
     </row>
@@ -2028,31 +2031,31 @@
         <v>4</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C10" s="7">
         <v>2451.8302696650185</v>
       </c>
       <c r="D10" s="8">
-        <v>0.77007517439812101</v>
+        <v>0.78896948195709271</v>
       </c>
       <c r="E10" s="9">
-        <v>46173</v>
+        <v>46264</v>
       </c>
       <c r="F10" s="1">
         <v>54</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H10" s="7">
-        <v>54.564803997650458</v>
+        <v>54.991363395254893</v>
       </c>
       <c r="I10" s="8">
-        <v>0.20941231245620498</v>
+        <v>0.22590722153566348</v>
       </c>
       <c r="J10" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="K10" s="7"/>
     </row>
@@ -2061,31 +2064,31 @@
         <v>5</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C11" s="7">
-        <v>2436.9693011103855</v>
+        <v>2437.0004043420113</v>
       </c>
       <c r="D11" s="8">
-        <v>0.78533537287481014</v>
+        <v>0.80637298300102289</v>
       </c>
       <c r="E11" s="9">
-        <v>46142</v>
+        <v>46234</v>
       </c>
       <c r="F11" s="1">
         <v>55</v>
       </c>
       <c r="G11" s="36" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H11" s="7">
-        <v>53.908121053777492</v>
+        <v>53.939224285403256</v>
       </c>
       <c r="I11" s="8">
-        <v>0.49371738631970125</v>
+        <v>0.51931070334444573</v>
       </c>
       <c r="J11" s="9">
-        <v>46173</v>
+        <v>46264</v>
       </c>
       <c r="K11" s="7"/>
     </row>
@@ -2094,31 +2097,31 @@
         <v>6</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C12" s="7">
-        <v>2346.4277938477808</v>
+        <v>2386.5509626450189</v>
       </c>
       <c r="D12" s="8">
-        <v>8.0220898295905715E-2</v>
+        <v>9.0804732373579042E-2</v>
       </c>
       <c r="E12" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="F12" s="1">
         <v>56</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H12" s="7">
-        <v>49.021793661161389</v>
+        <v>47.324045628440793</v>
       </c>
       <c r="I12" s="8">
-        <v>0.78773924693753528</v>
+        <v>0.78422400469407483</v>
       </c>
       <c r="J12" s="9">
-        <v>46173</v>
+        <v>46234</v>
       </c>
       <c r="K12" s="7"/>
     </row>
@@ -2127,31 +2130,31 @@
         <v>7</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C13" s="7">
-        <v>2282.9772013312186</v>
+        <v>2270.5359086809121</v>
       </c>
       <c r="D13" s="8">
-        <v>0.41371167324160585</v>
+        <v>0.44300699217402328</v>
       </c>
       <c r="E13" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="F13" s="1">
         <v>57</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H13" s="7">
-        <v>43.85555659232994</v>
+        <v>44.788653541102917</v>
       </c>
       <c r="I13" s="8">
-        <v>0.2579000490645007</v>
+        <v>4.9487322025276191E-2</v>
       </c>
       <c r="J13" s="9">
-        <v>46142</v>
+        <v>46264</v>
       </c>
       <c r="K13" s="7"/>
     </row>
@@ -2160,31 +2163,31 @@
         <v>8</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C14" s="7">
         <v>1039.9365494074837</v>
       </c>
       <c r="D14" s="8">
-        <v>0.12704420724841836</v>
+        <v>0.13703283927477111</v>
       </c>
       <c r="E14" s="9">
-        <v>46173</v>
+        <v>46234</v>
       </c>
       <c r="F14" s="1">
         <v>58</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H14" s="7">
         <v>43.85555659232994</v>
       </c>
       <c r="I14" s="8">
-        <v>4.2873301395072519E-2</v>
+        <v>0.28235271603604756</v>
       </c>
       <c r="J14" s="9">
-        <v>46203</v>
+        <v>46234</v>
       </c>
       <c r="K14" s="7"/>
     </row>
@@ -2193,31 +2196,31 @@
         <v>9</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C15" s="7">
         <v>880.52</v>
       </c>
       <c r="D15" s="8">
-        <v>0.16801358956054788</v>
+        <v>0.17141169916908189</v>
       </c>
       <c r="E15" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="F15" s="1">
         <v>59</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H15" s="7">
         <v>41.040714130198126</v>
       </c>
       <c r="I15" s="8">
-        <v>0.64100220868149949</v>
+        <v>0.66809403302568782</v>
       </c>
       <c r="J15" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="K15" s="7"/>
       <c r="M15" s="10"/>
@@ -2229,31 +2232,31 @@
         <v>10</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C16" s="7">
         <v>845.97309041709434</v>
       </c>
       <c r="D16" s="8">
-        <v>8.5053340082011555E-2</v>
+        <v>0.10277384150782244</v>
       </c>
       <c r="E16" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="F16" s="1">
         <v>60</v>
       </c>
       <c r="G16" s="36" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H16" s="7">
         <v>36.522495807891509</v>
       </c>
       <c r="I16" s="8">
-        <v>0.18666311942571792</v>
+        <v>0.20641038320285582</v>
       </c>
       <c r="J16" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K16" s="7"/>
     </row>
@@ -2262,28 +2265,28 @@
         <v>11</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C17" s="7">
-        <v>632.429473080153</v>
+        <v>647.98366638673758</v>
       </c>
       <c r="D17" s="8">
-        <v>0.27870010383598004</v>
+        <v>0.30899861773059312</v>
       </c>
       <c r="E17" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="F17" s="1">
         <v>61</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H17" s="7">
         <v>34.670153027899602</v>
       </c>
       <c r="I17" s="8">
-        <v>4.7556294325655633E-2</v>
+        <v>5.355634888695858E-2</v>
       </c>
       <c r="J17" s="9">
         <v>46053</v>
@@ -2295,31 +2298,31 @@
         <v>12</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C18" s="7">
         <v>612.45373394295666</v>
       </c>
       <c r="D18" s="8">
-        <v>0.70011775761981587</v>
+        <v>0.72678262532124316</v>
       </c>
       <c r="E18" s="9">
-        <v>46142</v>
+        <v>46234</v>
       </c>
       <c r="F18" s="1">
         <v>62</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H18" s="7">
         <v>31.694193026655469</v>
       </c>
       <c r="I18" s="8">
-        <v>0.23354082237196749</v>
+        <v>0.24541117316741665</v>
       </c>
       <c r="J18" s="9">
-        <v>46142</v>
+        <v>46234</v>
       </c>
       <c r="K18" s="7"/>
     </row>
@@ -2328,31 +2331,31 @@
         <v>13</v>
       </c>
       <c r="B19" s="36" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C19" s="7">
-        <v>530.62416799999994</v>
+        <v>532.09321380387655</v>
       </c>
       <c r="D19" s="8">
-        <v>0.5636700334017497</v>
+        <v>0.52868414484829696</v>
       </c>
       <c r="E19" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="F19" s="1">
         <v>63</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H19" s="7">
         <v>27.370843830674009</v>
       </c>
       <c r="I19" s="8">
-        <v>6.9122708228597368E-2</v>
+        <v>8.2554613269585811E-2</v>
       </c>
       <c r="J19" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="K19" s="7"/>
     </row>
@@ -2361,13 +2364,13 @@
         <v>14</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C20" s="7">
         <v>508.4134241547697</v>
       </c>
       <c r="D20" s="8">
-        <v>0.50022589674966489</v>
+        <v>0.53146918678180255</v>
       </c>
       <c r="E20" s="9">
         <v>46053</v>
@@ -2376,16 +2379,16 @@
         <v>64</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H20" s="7">
         <v>26.281072812665236</v>
       </c>
       <c r="I20" s="8">
-        <v>0.28195380892100352</v>
+        <v>0.32646284610291143</v>
       </c>
       <c r="J20" s="9">
-        <v>46173</v>
+        <v>46234</v>
       </c>
       <c r="K20" s="7"/>
     </row>
@@ -2394,31 +2397,31 @@
         <v>15</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C21" s="7">
-        <v>431.71285496563098</v>
+        <v>438.55556592329941</v>
       </c>
       <c r="D21" s="8">
-        <v>0.8747649839749384</v>
+        <v>0.89926907966508951</v>
       </c>
       <c r="E21" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="F21" s="1">
         <v>65</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H21" s="7">
         <v>25.8</v>
       </c>
       <c r="I21" s="8">
-        <v>0.16691622050769908</v>
+        <v>0.18504973888557888</v>
       </c>
       <c r="J21" s="9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="K21" s="7"/>
     </row>
@@ -2427,13 +2430,13 @@
         <v>16</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C22" s="7">
         <v>423.93704705918947</v>
       </c>
       <c r="D22" s="8">
-        <v>8.3477555576036894E-2</v>
+        <v>9.3564486966670232E-2</v>
       </c>
       <c r="E22" s="9">
         <v>46142</v>
@@ -2442,16 +2445,16 @@
         <v>66</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H22" s="7">
-        <v>24.4</v>
+        <v>25.2</v>
       </c>
       <c r="I22" s="8">
-        <v>0.36361939816837174</v>
+        <v>0.36137286865782892</v>
       </c>
       <c r="J22" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K22" s="7"/>
     </row>
@@ -2460,31 +2463,31 @@
         <v>17</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C23" s="7">
         <v>382.66305869179814</v>
       </c>
       <c r="D23" s="8">
-        <v>0.75744378389678535</v>
+        <v>0.80990974780262603</v>
       </c>
       <c r="E23" s="9">
-        <v>46142</v>
+        <v>46234</v>
       </c>
       <c r="F23" s="1">
         <v>67</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H23" s="7">
-        <v>22.3</v>
+        <v>24.3</v>
       </c>
       <c r="I23" s="8">
-        <v>0.8327089053432486</v>
+        <v>0.81473437104360935</v>
       </c>
       <c r="J23" s="9" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="K23" s="7"/>
     </row>
@@ -2493,31 +2496,31 @@
         <v>18</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C24" s="7">
-        <v>368.37605642126221</v>
+        <v>377.10696556872261</v>
       </c>
       <c r="D24" s="8">
-        <v>0.76561979918765077</v>
+        <v>0.78926229248543822</v>
       </c>
       <c r="E24" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="F24" s="1">
         <v>68</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H24" s="7">
-        <v>22.119496438679981</v>
+        <v>22.120811794345432</v>
       </c>
       <c r="I24" s="8">
-        <v>5.3918399652124346E-2</v>
+        <v>6.0355451050241003E-2</v>
       </c>
       <c r="J24" s="9">
-        <v>46173</v>
+        <v>46234</v>
       </c>
       <c r="K24" s="7"/>
     </row>
@@ -2526,31 +2529,31 @@
         <v>19</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C25" s="7">
         <v>323.06743180616468</v>
       </c>
       <c r="D25" s="8">
-        <v>7.8943992615318689E-2</v>
+        <v>8.847864183651781E-2</v>
       </c>
       <c r="E25" s="9">
-        <v>46173</v>
+        <v>46234</v>
       </c>
       <c r="F25" s="1">
         <v>69</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H25" s="7">
         <v>21.865850020217103</v>
       </c>
       <c r="I25" s="8">
-        <v>0.2551913738640561</v>
+        <v>0.27969524516354466</v>
       </c>
       <c r="J25" s="9" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K25" s="7"/>
     </row>
@@ -2559,31 +2562,31 @@
         <v>20</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C26" s="7">
         <v>310.28712260893911</v>
       </c>
       <c r="D26" s="8">
-        <v>0.18621192429727287</v>
+        <v>0.21183677678065688</v>
       </c>
       <c r="E26" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="F26" s="1">
         <v>70</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H26" s="7">
         <v>21.53504649933128</v>
       </c>
       <c r="I26" s="8">
-        <v>5.3986321990948286E-2</v>
+        <v>5.7507078403225935E-2</v>
       </c>
       <c r="J26" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="K26" s="7"/>
     </row>
@@ -2592,31 +2595,31 @@
         <v>21</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C27" s="7">
         <v>286.83400205281328</v>
       </c>
       <c r="D27" s="8">
-        <v>0.7907830950942667</v>
+        <v>0.81073482339912162</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F27" s="1">
         <v>71</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H27" s="7">
         <v>15.508071288606887</v>
       </c>
       <c r="I27" s="8">
-        <v>6.1223243320501233E-2</v>
+        <v>6.7944656204348669E-2</v>
       </c>
       <c r="J27" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="K27" s="7"/>
     </row>
@@ -2625,31 +2628,31 @@
         <v>22</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C28" s="7">
         <v>281.57755590805886</v>
       </c>
       <c r="D28" s="8">
-        <v>0.29473196295280824</v>
+        <v>0.32178816701014723</v>
       </c>
       <c r="E28" s="9">
-        <v>46142</v>
+        <v>46234</v>
       </c>
       <c r="F28" s="1">
         <v>72</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H28" s="7">
         <v>14.281469316662001</v>
       </c>
       <c r="I28" s="8">
-        <v>5.6122998023034582E-2</v>
+        <v>6.5793073219113402E-2</v>
       </c>
       <c r="J28" s="9">
-        <v>46203</v>
+        <v>46234</v>
       </c>
       <c r="K28" s="7"/>
     </row>
@@ -2658,31 +2661,31 @@
         <v>23</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C29" s="7">
         <v>280.05349755839632</v>
       </c>
       <c r="D29" s="8">
-        <v>0.71333663244407763</v>
+        <v>0.73963703697651051</v>
       </c>
       <c r="E29" s="9">
-        <v>46203</v>
+        <v>46234</v>
       </c>
       <c r="F29" s="1">
         <v>73</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="H29" s="7">
         <v>13.872041305091599</v>
       </c>
       <c r="I29" s="8">
-        <v>0.64407872727387361</v>
+        <v>0.66761502434710351</v>
       </c>
       <c r="J29" s="9">
-        <v>46203</v>
+        <v>46234</v>
       </c>
       <c r="K29" s="7"/>
     </row>
@@ -2691,28 +2694,28 @@
         <v>24</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C30" s="7">
         <v>234.51836645827501</v>
       </c>
       <c r="D30" s="8">
-        <v>0.1086788056977743</v>
+        <v>0.12114482320964652</v>
       </c>
       <c r="E30" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="F30" s="1">
         <v>74</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="H30" s="7">
         <v>13.16159831</v>
       </c>
       <c r="I30" s="8">
-        <v>0.51952186927675437</v>
+        <v>0.550642491251493</v>
       </c>
       <c r="J30" s="9">
         <v>45930</v>
@@ -2724,31 +2727,31 @@
         <v>25</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C31" s="7">
         <v>227.39572641597462</v>
       </c>
       <c r="D31" s="8">
-        <v>0.54992027233582264</v>
+        <v>0.57823126859636909</v>
       </c>
       <c r="E31" s="9">
-        <v>46203</v>
+        <v>46234</v>
       </c>
       <c r="F31" s="1">
         <v>75</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H31" s="7">
         <v>13.063357282821686</v>
       </c>
       <c r="I31" s="8">
-        <v>0.60826506749603682</v>
+        <v>0.63764680046117683</v>
       </c>
       <c r="J31" s="9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="K31" s="7"/>
     </row>
@@ -2757,31 +2760,31 @@
         <v>26</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C32" s="7">
-        <v>203.68750583185593</v>
+        <v>203.40959845727971</v>
       </c>
       <c r="D32" s="8">
-        <v>5.9013740052141231E-2</v>
+        <v>6.5297345910829432E-2</v>
       </c>
       <c r="E32" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="F32" s="1">
         <v>76</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="H32" s="7">
         <v>12.416410065005755</v>
       </c>
       <c r="I32" s="8">
-        <v>0.14605653521137224</v>
+        <v>0.17756076866448811</v>
       </c>
       <c r="J32" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="K32" s="7"/>
     </row>
@@ -2790,7 +2793,7 @@
         <v>27</v>
       </c>
       <c r="B33" s="36" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C33" s="7">
         <v>178.1</v>
@@ -2805,16 +2808,16 @@
         <v>77</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="H33" s="7">
         <v>12.03695063917141</v>
       </c>
       <c r="I33" s="8">
-        <v>0.11627662611681167</v>
+        <v>0.12757176727830044</v>
       </c>
       <c r="J33" s="9">
-        <v>46142</v>
+        <v>46234</v>
       </c>
       <c r="K33" s="7"/>
     </row>
@@ -2823,31 +2826,31 @@
         <v>28</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C34" s="7">
-        <v>174.61354234704987</v>
+        <v>175.63994899070013</v>
       </c>
       <c r="D34" s="8">
-        <v>0.23138992435245018</v>
+        <v>0.28586659532734909</v>
       </c>
       <c r="E34" s="9">
-        <v>45991</v>
+        <v>46203</v>
       </c>
       <c r="F34" s="1">
         <v>78</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H34" s="7">
-        <v>9.1754533296009448</v>
+        <v>9.7944076389536878</v>
       </c>
       <c r="I34" s="8">
-        <v>0.34842034747581563</v>
+        <v>2.7611666378939904E-2</v>
       </c>
       <c r="J34" s="9">
-        <v>46022</v>
+        <v>46203</v>
       </c>
       <c r="K34" s="7"/>
     </row>
@@ -2856,31 +2859,31 @@
         <v>29</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C35" s="7">
         <v>173.55603247177382</v>
       </c>
       <c r="D35" s="8">
-        <v>0.33577703476482945</v>
+        <v>0.37620415896119819</v>
       </c>
       <c r="E35" s="9">
-        <v>46173</v>
+        <v>46234</v>
       </c>
       <c r="F35" s="1">
         <v>79</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H35" s="7">
-        <v>8.3947622157942199</v>
+        <v>9.1754533296009448</v>
       </c>
       <c r="I35" s="8">
-        <v>2.1527974505022567E-2</v>
+        <v>0.37734088055322018</v>
       </c>
       <c r="J35" s="9">
-        <v>46112</v>
+        <v>46022</v>
       </c>
       <c r="K35" s="7"/>
     </row>
@@ -2889,28 +2892,28 @@
         <v>30</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C36" s="7">
-        <v>172.44498531926195</v>
+        <v>172.44498531926567</v>
       </c>
       <c r="D36" s="8">
-        <v>6.0731590361504266E-2</v>
+        <v>6.7756384925343638E-2</v>
       </c>
       <c r="E36" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="F36" s="1">
         <v>80</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H36" s="7">
         <v>8.193368791017388</v>
       </c>
       <c r="I36" s="8">
-        <v>0.10566132238915399</v>
+        <v>0.11808344941125251</v>
       </c>
       <c r="J36" s="9">
         <v>45991</v>
@@ -2922,28 +2925,28 @@
         <v>31</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C37" s="7">
         <v>161.22049080899507</v>
       </c>
       <c r="D37" s="8">
-        <v>0.91530559524129385</v>
+        <v>0.92451590054620925</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F37" s="1">
         <v>81</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H37" s="7">
         <v>7.9877242387484069</v>
       </c>
       <c r="I37" s="8">
-        <v>4.9205949282273953E-2</v>
+        <v>5.5402029814725751E-2</v>
       </c>
       <c r="J37" s="9">
         <v>46022</v>
@@ -2955,13 +2958,13 @@
         <v>32</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C38" s="7">
         <v>146.6517371154863</v>
       </c>
       <c r="D38" s="8">
-        <v>0.18612558090239356</v>
+        <v>0.20583036918211572</v>
       </c>
       <c r="E38" s="9">
         <v>46142</v>
@@ -2970,13 +2973,13 @@
         <v>82</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="H38" s="7">
         <v>7.8803943889770158</v>
       </c>
       <c r="I38" s="8">
-        <v>0.15821000422619425</v>
+        <v>0.17559705442996981</v>
       </c>
       <c r="J38" s="9">
         <v>46053</v>
@@ -2990,31 +2993,31 @@
         <v>33</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C39" s="7">
-        <v>133.51727650772915</v>
+        <v>133.52467425585519</v>
       </c>
       <c r="D39" s="8">
-        <v>0.16485864617044299</v>
+        <v>0.18597396177078176</v>
       </c>
       <c r="E39" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="F39" s="1">
         <v>83</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H39" s="7">
-        <v>7.8336409442941131</v>
+        <v>7.833640788777954</v>
       </c>
       <c r="I39" s="8">
-        <v>0.14239466848466009</v>
+        <v>0.14118809217302114</v>
       </c>
       <c r="J39" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="K39" s="7"/>
       <c r="M39" s="7"/>
@@ -3025,31 +3028,31 @@
         <v>34</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C40" s="7">
-        <v>129.66764921775373</v>
+        <v>129.91579515411652</v>
       </c>
       <c r="D40" s="8">
-        <v>0.32018011573420296</v>
+        <v>0.35016141276119417</v>
       </c>
       <c r="E40" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="F40" s="1">
         <v>84</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H40" s="7">
         <v>7.4152564461431689</v>
       </c>
       <c r="I40" s="8">
-        <v>0.18213918826617315</v>
+        <v>0.20152644515519416</v>
       </c>
       <c r="J40" s="9" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="K40" s="7"/>
       <c r="M40" s="7"/>
@@ -3060,31 +3063,31 @@
         <v>35</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C41" s="7">
         <v>125.71926223134584</v>
       </c>
       <c r="D41" s="8">
-        <v>0.22228347543295884</v>
+        <v>0.24416176853229615</v>
       </c>
       <c r="E41" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="F41" s="1">
         <v>85</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="H41" s="7">
-        <v>6.893533491953594</v>
+        <v>6.8935359491088928</v>
       </c>
       <c r="I41" s="8">
-        <v>0.15842218933504626</v>
+        <v>0.17049301146438045</v>
       </c>
       <c r="J41" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="K41" s="7"/>
       <c r="N41" s="15"/>
@@ -3094,28 +3097,28 @@
         <v>36</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C42" s="7">
         <v>125.53264284159123</v>
       </c>
       <c r="D42" s="8">
-        <v>0.21928303596441839</v>
+        <v>0.24110774841008564</v>
       </c>
       <c r="E42" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="F42" s="1">
         <v>86</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H42" s="7">
         <v>6.8427109576685021</v>
       </c>
       <c r="I42" s="8">
-        <v>9.3924136161714383E-2</v>
+        <v>0.10512857935131645</v>
       </c>
       <c r="J42" s="9">
         <v>45961</v>
@@ -3129,31 +3132,31 @@
         <v>37</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C43" s="7">
         <v>120.04396420065473</v>
       </c>
       <c r="D43" s="8">
-        <v>5.7273863711560812E-2</v>
+        <v>6.6210968607057705E-2</v>
       </c>
       <c r="E43" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="F43" s="1">
         <v>87</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="H43" s="7">
         <v>6.7275978974215418</v>
       </c>
       <c r="I43" s="8">
-        <v>4.5458389444432298E-2</v>
+        <v>5.120798764471423E-2</v>
       </c>
       <c r="J43" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K43" s="7"/>
       <c r="M43" s="7"/>
@@ -3164,31 +3167,31 @@
         <v>38</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C44" s="7">
-        <v>115.23309106385524</v>
+        <v>115.24712547845604</v>
       </c>
       <c r="D44" s="8">
-        <v>0.27498715186431927</v>
+        <v>0.27491590057916465</v>
       </c>
       <c r="E44" s="9">
-        <v>46173</v>
+        <v>46264</v>
       </c>
       <c r="F44" s="1">
         <v>88</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="H44" s="7">
         <v>6.6560915679139061</v>
       </c>
       <c r="I44" s="8">
-        <v>0.14091737239396418</v>
+        <v>0.15859414789683912</v>
       </c>
       <c r="J44" s="9">
-        <v>46142</v>
+        <v>46234</v>
       </c>
       <c r="K44" s="7"/>
       <c r="M44" s="7"/>
@@ -3199,31 +3202,31 @@
         <v>39</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C45" s="7">
         <v>114.73982146745047</v>
       </c>
       <c r="D45" s="8">
-        <v>0.65154768139639263</v>
+        <v>0.69453587273452622</v>
       </c>
       <c r="E45" s="9">
-        <v>46142</v>
+        <v>46234</v>
       </c>
       <c r="F45" s="1">
         <v>89</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="H45" s="7">
         <v>5.8163043140182262</v>
       </c>
       <c r="I45" s="8">
-        <v>0.10463586584222238</v>
+        <v>0.11728396456025017</v>
       </c>
       <c r="J45" s="9">
-        <v>46173</v>
+        <v>46203</v>
       </c>
       <c r="K45" s="7"/>
       <c r="M45" s="7"/>
@@ -3234,31 +3237,31 @@
         <v>40</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C46" s="7">
         <v>110.01213026033405</v>
       </c>
       <c r="D46" s="8">
-        <v>0.20711130070332562</v>
+        <v>0.21787303442722319</v>
       </c>
       <c r="E46" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="F46" s="1">
         <v>90</v>
       </c>
       <c r="G46" s="36" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H46" s="7">
         <v>4.7460732170072477</v>
       </c>
       <c r="I46" s="35" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J46" s="9">
-        <v>46173</v>
+        <v>46234</v>
       </c>
       <c r="K46" s="7"/>
     </row>
@@ -3267,28 +3270,28 @@
         <v>41</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C47" s="7">
         <v>104.44677475039657</v>
       </c>
       <c r="D47" s="8">
-        <v>3.1090262955461991E-2</v>
+        <v>3.5038544742709614E-2</v>
       </c>
       <c r="E47" s="9">
-        <v>46203</v>
+        <v>46234</v>
       </c>
       <c r="F47" s="1">
         <v>91</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="H47" s="7">
         <v>4.6750246648626792</v>
       </c>
       <c r="I47" s="8">
-        <v>9.14834655007353E-3</v>
+        <v>1.0355255094242836E-2</v>
       </c>
       <c r="J47" s="9">
         <v>46053</v>
@@ -3300,28 +3303,28 @@
         <v>42</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C48" s="7">
         <v>103.62041616123916</v>
       </c>
       <c r="D48" s="8">
-        <v>0.15637066768266664</v>
+        <v>0.16807555412795858</v>
       </c>
       <c r="E48" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="F48" s="1">
         <v>92</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="H48" s="7">
         <v>4.6654847438648872</v>
       </c>
       <c r="I48" s="8">
-        <v>9.177666826962716E-2</v>
+        <v>0.10275398654234807</v>
       </c>
       <c r="J48" s="9">
         <v>46112</v>
@@ -3333,31 +3336,31 @@
         <v>43</v>
       </c>
       <c r="B49" s="36" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C49" s="7">
         <v>102</v>
       </c>
       <c r="D49" s="35" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E49" s="9">
-        <v>45382</v>
+        <v>46112</v>
       </c>
       <c r="F49" s="1">
         <v>93</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H49" s="7">
-        <v>4.5460241741357343</v>
+        <v>4.5700302873571896</v>
       </c>
       <c r="I49" s="8">
-        <v>0.11545062437947065</v>
+        <v>0.40874912658894935</v>
       </c>
       <c r="J49" s="9">
-        <v>46081</v>
+        <v>46203</v>
       </c>
       <c r="K49" s="7"/>
       <c r="L49" s="18"/>
@@ -3367,31 +3370,31 @@
         <v>44</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C50" s="7">
-        <v>87.089048552144561</v>
+        <v>87.053177848278438</v>
       </c>
       <c r="D50" s="8">
-        <v>7.743435987553815E-2</v>
+        <v>8.6973157832745673E-2</v>
       </c>
       <c r="E50" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="F50" s="1">
         <v>94</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="H50" s="7">
-        <v>4.4352814123663657</v>
+        <v>4.5460241741357343</v>
       </c>
       <c r="I50" s="8">
-        <v>0.42927610772015318</v>
+        <v>0.12885781432973631</v>
       </c>
       <c r="J50" s="9">
-        <v>46112</v>
+        <v>46081</v>
       </c>
       <c r="K50" s="7"/>
       <c r="L50" s="18"/>
@@ -3401,31 +3404,31 @@
         <v>45</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C51" s="7">
-        <v>82.428726944729561</v>
+        <v>85.759758638922577</v>
       </c>
       <c r="D51" s="8">
-        <v>5.9431020606765715E-2</v>
+        <v>6.8182467875945882E-2</v>
       </c>
       <c r="E51" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="F51" s="1">
         <v>95</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="H51" s="7">
         <v>4.2300395011041649</v>
       </c>
       <c r="I51" s="8">
-        <v>0.15511705224166628</v>
+        <v>0.17176070339817343</v>
       </c>
       <c r="J51" s="9">
-        <v>46203</v>
+        <v>46234</v>
       </c>
       <c r="K51" s="7"/>
     </row>
@@ -3434,31 +3437,31 @@
         <v>46</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C52" s="7">
         <v>79.87309881496688</v>
       </c>
       <c r="D52" s="8">
-        <v>0.15208215968376607</v>
+        <v>0.16009023336661068</v>
       </c>
       <c r="E52" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="F52" s="1">
         <v>96</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="H52" s="7">
-        <v>3.9368848412180029</v>
+        <v>3.7323877950919102</v>
       </c>
       <c r="I52" s="8">
-        <v>0.12156584273284984</v>
+        <v>5.8111474399852363E-2</v>
       </c>
       <c r="J52" s="9">
-        <v>45869</v>
+        <v>46234</v>
       </c>
       <c r="K52" s="7"/>
       <c r="L52" s="18"/>
@@ -3468,31 +3471,31 @@
         <v>47</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C53" s="7">
-        <v>78.977297968958979</v>
+        <v>78.989739572641597</v>
       </c>
       <c r="D53" s="8">
-        <v>0.2095592088962131</v>
+        <v>0.25197217354501095</v>
       </c>
       <c r="E53" s="9">
-        <v>46173</v>
+        <v>46234</v>
       </c>
       <c r="F53" s="1">
         <v>97</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H53" s="7">
-        <v>3.7323877950919102</v>
+        <v>3.4835619420857831</v>
       </c>
       <c r="I53" s="8">
-        <v>5.6375973874119224E-2</v>
-      </c>
-      <c r="J53" s="9">
-        <v>46081</v>
+        <v>5.3812020904150167E-2</v>
+      </c>
+      <c r="J53" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="K53" s="7"/>
       <c r="L53" s="18"/>
@@ -3502,31 +3505,31 @@
         <v>48</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C54" s="7">
-        <v>78.724697707691831</v>
+        <v>74.981729806018166</v>
       </c>
       <c r="D54" s="8">
-        <v>0.37884911396033444</v>
+        <v>4.2142021602783269E-2</v>
       </c>
       <c r="E54" s="9">
-        <v>46203</v>
+        <v>46234</v>
       </c>
       <c r="F54" s="1">
         <v>98</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="H54" s="7">
-        <v>3.4835619420857831</v>
+        <v>3.1103231625765919</v>
       </c>
       <c r="I54" s="8">
-        <v>4.7784768933090124E-2</v>
-      </c>
-      <c r="J54" s="9" t="s">
-        <v>26</v>
+        <v>0.16982704142646449</v>
+      </c>
+      <c r="J54" s="9">
+        <v>46173</v>
       </c>
       <c r="K54" s="7"/>
       <c r="L54" s="18"/>
@@ -3536,31 +3539,31 @@
         <v>49</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C55" s="7">
-        <v>74.963647939953034</v>
+        <v>74.647755901838195</v>
       </c>
       <c r="D55" s="8">
-        <v>3.5208825415738471E-2</v>
+        <v>0.37318770329312301</v>
       </c>
       <c r="E55" s="9">
-        <v>46142</v>
+        <v>46264</v>
       </c>
       <c r="F55" s="1">
         <v>99</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="H55" s="7">
-        <v>3.1103231625765919</v>
+        <v>2.239432677055146</v>
       </c>
       <c r="I55" s="8">
-        <v>0.15290535266720154</v>
+        <v>0.10718466969005086</v>
       </c>
       <c r="J55" s="9">
-        <v>46173</v>
+        <v>46234</v>
       </c>
       <c r="K55" s="7"/>
       <c r="L55" s="18"/>
@@ -3570,31 +3573,31 @@
         <v>50</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C56" s="7">
         <v>66.548474386488763</v>
       </c>
       <c r="D56" s="8">
-        <v>6.7978513736335885E-2</v>
+        <v>7.6764381612016847E-2</v>
       </c>
       <c r="E56" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="F56" s="1">
         <v>100</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="H56" s="7">
-        <v>2.239432677055146</v>
+        <v>2.0964508102391837</v>
       </c>
       <c r="I56" s="8">
-        <v>9.5483745670142228E-2</v>
+        <v>5.7173442743201588E-2</v>
       </c>
       <c r="J56" s="9">
-        <v>46142</v>
+        <v>46264</v>
       </c>
       <c r="K56" s="7"/>
       <c r="L56" s="18"/>
@@ -3646,7 +3649,7 @@
     </row>
     <row r="61" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="34" t="s">
-        <v>109</v>
+        <v>7</v>
       </c>
       <c r="B61" s="34"/>
       <c r="C61" s="34"/>
@@ -3698,16 +3701,16 @@
     <row r="64" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A64" s="3"/>
       <c r="B64" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C64" s="24">
-        <v>36705.428444182769</v>
+        <v>36888.970556925138</v>
       </c>
       <c r="D64" s="25">
-        <v>0.2503475199865412</v>
+        <v>0.27527666835625447</v>
       </c>
       <c r="E64" s="9">
-        <v>46173</v>
+        <v>46234</v>
       </c>
       <c r="F64" s="3"/>
       <c r="G64" s="22"/>
@@ -3722,13 +3725,13 @@
         <v>6</v>
       </c>
       <c r="C65" s="19">
-        <v>10807.635687847969</v>
+        <v>10807.480171689842</v>
       </c>
       <c r="D65" s="25">
-        <v>0.69877452540624663</v>
+        <v>0.72461846039301392</v>
       </c>
       <c r="E65" s="9">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="F65" s="3"/>
       <c r="H65" s="19"/>
@@ -4244,28 +4247,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="81ba2d26-7208-4098-b7cd-1db435ad554f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TranslatedLang xmlns="81ba2d26-7208-4098-b7cd-1db435ad554f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A4383A4629DC9B4D859E49C7E0774F94" ma:contentTypeVersion="21" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="56bf5c403728eecf3266d4d4ea73af37">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="81ba2d26-7208-4098-b7cd-1db435ad554f" xmlns:ns3="d6c5908d-f417-492b-af08-ab5b835958da" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8d393ea0eeffda1ff0d47238829003b1" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -4537,27 +4518,30 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A779781-46C7-48D1-B059-4004BD4509BD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="81ba2d26-7208-4098-b7cd-1db435ad554f"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="81ba2d26-7208-4098-b7cd-1db435ad554f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TranslatedLang xmlns="81ba2d26-7208-4098-b7cd-1db435ad554f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{11B4DC92-66E7-4F23-8B9A-966783F0B2C9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C676504B-D7FB-4449-AD7A-36C9800350A2}">
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A8D1E86F-7150-40B8-913A-6DC54005BA99}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
@@ -4576,6 +4560,25 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1D7C052-1AC1-4918-A0D7-960F3D964B9B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="81ba2d26-7208-4098-b7cd-1db435ad554f"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FDC0CF33-EAC4-4408-B8B5-8BBB1E7CCBD2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{49a08eac-c57e-4d52-9fcb-029f5cb8627d}" enabled="0" method="" siteId="{49a08eac-c57e-4d52-9fcb-029f5cb8627d}" removed="1"/>

</xml_diff>